<commit_message>
Scope LW rent waiver: diagnostic Current column keeps GL 6% occupancy
The rent waiver was already correctly gated in the scenarios (booked
occupancy through July, waived from the 8/1 go-live and all of 2027).
Fix the one leak: the LW P&L current-vs-adjusted tab's Current column
now holds GL ~6% occupancy instead of following the waived input, so
current economics read correctly. Daypart sensitivity keep-rate
updated 62.5c -> 68.5c (rent no longer applies to incremental
revenue).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VCQW3YoSqaJfwSKLPDyQy8
</commit_message>
<xml_diff>
--- a/Method_Operating_Model_2027_14.xlsx
+++ b/Method_Operating_Model_2027_14.xlsx
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1435" uniqueCount="561">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1435" uniqueCount="562">
   <si>
     <t xml:space="preserve">Method Terrapin</t>
   </si>
@@ -900,7 +900,10 @@
     <t xml:space="preserve">Change</t>
   </si>
   <si>
-    <t xml:space="preserve">Both columns at base revenue (no pricing/retail uplift) and go-forward owner terms (4% fee + 6% rent) — the gap isolates the labor model. Current labor from GL roles (LW Labor Model); Adjusted = single 6am–4pm shift + wknd 2nd barista + BOH cook kept.</t>
+    <t xml:space="preserve">Occupancy Cost  (Current: GL ~6% · Adjusted: waived)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Both columns at base revenue (no pricing/retail uplift). Current column carries GL-style terms (6% occupancy, GL CC); Adjusted column carries go-forward terms (4% fee, rent waived, 2.5% CC) plus the single-shift labor model with BOH cook kept.</t>
   </si>
   <si>
     <t xml:space="preserve">Profit &amp; Loss Budget — annualized 2026 Modified run-rate (Dec-2026 forecast base · all levers in effect)</t>
@@ -1254,7 +1257,7 @@
     <t xml:space="preserve">Lost revenue / yr</t>
   </si>
   <si>
-    <t xml:space="preserve">NOP impact / yr  (× 62.5¢ keep-rate: ~25% COGS · 2.5% CC · 4% fee · 6% rent)</t>
+    <t xml:space="preserve">NOP impact / yr  (× 68.5¢ keep-rate: ~25% COGS · 2.5% CC · 4% fee · rent waived)</t>
   </si>
   <si>
     <t xml:space="preserve">Grid — NOP impact at 25% / 50% / 75% / 100% loss:</t>
@@ -20420,15 +20423,15 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="19" t="s">
-        <v>75</v>
+        <v>286</v>
       </c>
       <c r="C54" s="20" t="n">
-        <f aca="false">C20*'LW Assumptions'!$C$41</f>
-        <v>0</v>
+        <f aca="false">C20*0.06</f>
+        <v>15972.1212</v>
       </c>
       <c r="D54" s="31" t="n">
         <f aca="false">IFERROR(C54/C$20,0)</f>
-        <v>0</v>
+        <v>0.06</v>
       </c>
       <c r="F54" s="20" t="n">
         <f aca="false">F20*'LW Assumptions'!$C$41</f>
@@ -20440,11 +20443,11 @@
       </c>
       <c r="I54" s="20" t="n">
         <f aca="false">F54-C54</f>
-        <v>0</v>
+        <v>-15972.1212</v>
       </c>
       <c r="J54" s="31" t="n">
         <f aca="false">IFERROR(I54/C54,0)</f>
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20592,11 +20595,11 @@
       </c>
       <c r="C60" s="24" t="n">
         <f aca="false">SUM(C53:C59)</f>
-        <v>16305.0808</v>
+        <v>32277.202</v>
       </c>
       <c r="D60" s="32" t="n">
         <f aca="false">IFERROR(C60/C$20,0)</f>
-        <v>0.0612507778866592</v>
+        <v>0.121250777886659</v>
       </c>
       <c r="F60" s="24" t="n">
         <f aca="false">SUM(F53:F59)</f>
@@ -20608,11 +20611,11 @@
       </c>
       <c r="I60" s="24" t="n">
         <f aca="false">F60-C60</f>
-        <v>0</v>
+        <v>-15972.1212</v>
       </c>
       <c r="J60" s="32" t="n">
         <f aca="false">IFERROR(I60/C60,0)</f>
-        <v>0</v>
+        <v>-0.494842186134969</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20621,11 +20624,11 @@
       </c>
       <c r="C62" s="24" t="n">
         <f aca="false">C41-C50-C60</f>
-        <v>-95580.407156</v>
+        <v>-111552.528356</v>
       </c>
       <c r="D62" s="32" t="n">
         <f aca="false">IFERROR(C62/C$20,0)</f>
-        <v>-0.359052148274457</v>
+        <v>-0.419052148274457</v>
       </c>
       <c r="F62" s="24" t="n">
         <f aca="false">F41-F50-F60</f>
@@ -20637,11 +20640,11 @@
       </c>
       <c r="I62" s="24" t="n">
         <f aca="false">F62-C62</f>
-        <v>60483.4295</v>
+        <v>76455.5507</v>
       </c>
       <c r="J62" s="32" t="n">
         <f aca="false">IFERROR(I62/C62,0)</f>
-        <v>-0.632801546882751</v>
+        <v>-0.685377120776732</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20677,11 +20680,11 @@
       </c>
       <c r="C66" s="33" t="n">
         <f aca="false">C62-C64</f>
-        <v>-95580.407156</v>
+        <v>-111552.528356</v>
       </c>
       <c r="D66" s="34" t="n">
         <f aca="false">IFERROR(C66/C$20,0)</f>
-        <v>-0.359052148274457</v>
+        <v>-0.419052148274457</v>
       </c>
       <c r="F66" s="33" t="n">
         <f aca="false">F62-F64</f>
@@ -20693,11 +20696,11 @@
       </c>
       <c r="I66" s="33" t="n">
         <f aca="false">F66-C66</f>
-        <v>60483.4295</v>
+        <v>76455.5507</v>
       </c>
       <c r="J66" s="34" t="n">
         <f aca="false">IFERROR(I66/C66,0)</f>
-        <v>-0.632801546882751</v>
+        <v>-0.685377120776732</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20760,11 +20763,11 @@
       </c>
       <c r="C70" s="35" t="n">
         <f aca="false">C66-C68-C69</f>
-        <v>-95580.407156</v>
+        <v>-111552.528356</v>
       </c>
       <c r="D70" s="36" t="n">
         <f aca="false">IFERROR(C70/C$20,0)</f>
-        <v>-0.359052148274457</v>
+        <v>-0.419052148274457</v>
       </c>
       <c r="F70" s="35" t="n">
         <f aca="false">F66-F68-F69</f>
@@ -20776,16 +20779,16 @@
       </c>
       <c r="I70" s="35" t="n">
         <f aca="false">F70-C70</f>
-        <v>60483.4295</v>
+        <v>76455.5507</v>
       </c>
       <c r="J70" s="36" t="n">
         <f aca="false">IFERROR(I70/C70,0)</f>
-        <v>-0.632801546882751</v>
+        <v>-0.685377120776732</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="13" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
   </sheetData>
@@ -20854,7 +20857,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26055,28 +26058,28 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="13" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="23" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="23" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C75" s="23" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E75" s="23" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="19" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C76" s="71" t="n">
         <f aca="false">'LW Assumptions'!$C$20+'LW Assumptions'!$C$21</f>
@@ -26089,7 +26092,7 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="19" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C77" s="71" t="n">
         <v>8</v>
@@ -26101,7 +26104,7 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="19" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C78" s="71" t="n">
         <v>13.5</v>
@@ -26113,7 +26116,7 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="19" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C79" s="71" t="n">
         <v>16</v>
@@ -26182,7 +26185,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="39" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B1" s="39"/>
       <c r="C1" s="39"/>
@@ -26194,7 +26197,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="40" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B2" s="40"/>
       <c r="C2" s="40"/>
@@ -26206,35 +26209,35 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="41" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="F4" s="41" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="72" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C5" s="42" t="s">
         <v>184</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="F5" s="72" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="G5" s="42" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="H5" s="42" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="46" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C6" s="49" t="n">
         <v>42998</v>
@@ -26244,7 +26247,7 @@
         <v>0.161523943357004</v>
       </c>
       <c r="F6" s="46" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="G6" s="49" t="n">
         <v>72907</v>
@@ -26256,7 +26259,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="46" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C7" s="49" t="n">
         <v>54634</v>
@@ -26266,7 +26269,7 @@
         <v>0.205235106780933</v>
       </c>
       <c r="F7" s="46" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="G7" s="49" t="n">
         <v>32396</v>
@@ -26278,7 +26281,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="46" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C8" s="49" t="n">
         <v>30727</v>
@@ -26288,7 +26291,7 @@
         <v>0.115427373541343</v>
       </c>
       <c r="F8" s="81" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="G8" s="44" t="n">
         <f aca="false">G6+G7</f>
@@ -26301,7 +26304,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="46" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C9" s="49" t="n">
         <v>12880</v>
@@ -26313,7 +26316,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="46" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C10" s="49" t="n">
         <v>886</v>
@@ -26323,12 +26326,12 @@
         <v>0.00332829931192859</v>
       </c>
       <c r="F10" s="62" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="46" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C11" s="49" t="n">
         <v>22733</v>
@@ -26338,12 +26341,12 @@
         <v>0.0853975488240097</v>
       </c>
       <c r="F11" s="62" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="81" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C12" s="44" t="n">
         <f aca="false">SUM(C6:C11)</f>
@@ -26354,17 +26357,17 @@
         <v>0.619296577839642</v>
       </c>
       <c r="F12" s="62" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="41" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="46" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C15" s="82" t="n">
         <f aca="false">'LW Assumptions'!C20+'LW Assumptions'!C21</f>
@@ -26373,7 +26376,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="46" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C16" s="53" t="n">
         <f aca="false">('LW Assumptions'!C20+'LW Assumptions'!C21)*'LW Assumptions'!C22*52</f>
@@ -26382,7 +26385,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="46" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C17" s="49" t="n">
         <f aca="false">C16*'LW Assumptions'!C23</f>
@@ -26391,7 +26394,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="46" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C18" s="49" t="n">
         <f aca="false">'LW Assumptions'!C26*52</f>
@@ -26400,7 +26403,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="46" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C19" s="49" t="n">
         <f aca="false">(C17+C18)*'LW Assumptions'!C24</f>
@@ -26409,7 +26412,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="46" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C20" s="53" t="n">
         <f aca="false">C17+C18+C19</f>
@@ -26418,7 +26421,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="83" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C21" s="84" t="n">
         <f aca="false">C12-C20</f>
@@ -26427,7 +26430,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="59" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C23" s="59"/>
       <c r="D23" s="59"/>
@@ -26476,7 +26479,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="85" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B1" s="37"/>
       <c r="C1" s="37"/>
@@ -26484,7 +26487,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="86" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B2" s="86"/>
       <c r="C2" s="86"/>
@@ -26493,18 +26496,18 @@
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="72"/>
       <c r="B4" s="42" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C4" s="42" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D4" s="42" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="81" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B5" s="87"/>
       <c r="C5" s="87"/>
@@ -26512,10 +26515,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="88" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B6" s="89" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C6" s="89" t="n">
         <f aca="false">'LW Assumptions'!$C$20+'LW Assumptions'!$C$21</f>
@@ -26524,7 +26527,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="88" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B7" s="90" t="n">
         <v>7</v>
@@ -26536,7 +26539,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="81" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B9" s="87"/>
       <c r="C9" s="87"/>
@@ -26544,7 +26547,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="88" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B10" s="91" t="n">
         <v>111.8</v>
@@ -26556,7 +26559,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="88" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B11" s="91" t="n">
         <v>13.3</v>
@@ -26568,7 +26571,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="92" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B12" s="93" t="n">
         <v>125.1</v>
@@ -26585,7 +26588,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="81" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B14" s="87"/>
       <c r="C14" s="87"/>
@@ -26593,7 +26596,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="88" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B15" s="96" t="n">
         <v>2207</v>
@@ -26605,7 +26608,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="88" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B16" s="96" t="n">
         <v>296</v>
@@ -26617,7 +26620,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="94" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B17" s="74" t="n">
         <v>2503</v>
@@ -26629,7 +26632,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="88" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B18" s="96" t="n">
         <f aca="false">'LW Assumptions'!$C$45/52</f>
@@ -26642,7 +26645,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="88" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B19" s="96" t="n">
         <f aca="false">(B17+B18)*'LW Assumptions'!$C$24</f>
@@ -26655,7 +26658,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="97" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B20" s="98" t="n">
         <f aca="false">B17+B18+B19</f>
@@ -26678,7 +26681,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="94" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B22" s="74" t="n">
         <f aca="false">B20*52</f>
@@ -26701,7 +26704,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="81" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B24" s="87"/>
       <c r="C24" s="87"/>
@@ -26709,7 +26712,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="88" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B25" s="96" t="n">
         <v>5888.94</v>
@@ -26720,7 +26723,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="94" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B26" s="101" t="n">
         <f aca="false">B20/B25</f>
@@ -26743,7 +26746,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="102" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B28" s="102"/>
       <c r="C28" s="102"/>
@@ -26751,7 +26754,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="94" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C29" s="74" t="n">
         <f aca="false">B20-C20</f>
@@ -26764,12 +26767,12 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="103" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="104" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B32" s="104"/>
       <c r="C32" s="104"/>
@@ -26783,12 +26786,12 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="103" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="104" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B36" s="104"/>
       <c r="C36" s="104"/>
@@ -26802,12 +26805,12 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="105" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="104" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B40" s="104"/>
       <c r="C40" s="104"/>
@@ -26858,24 +26861,24 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B4" s="14"/>
       <c r="C4" s="14" t="s">
         <v>119</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="C5" s="20" t="n">
         <v>2411</v>
@@ -26887,7 +26890,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C6" s="20" t="n">
         <v>89592</v>
@@ -26899,7 +26902,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C7" s="20" t="n">
         <v>13203</v>
@@ -26911,7 +26914,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="19" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="C8" s="33" t="n">
         <v>27886</v>
@@ -26923,7 +26926,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="23" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C9" s="24" t="n">
         <f aca="false">SUM(C5:C8)</f>
@@ -26932,22 +26935,22 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B12" s="14"/>
       <c r="C12" s="14" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27042,27 +27045,27 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="14" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B21" s="14"/>
       <c r="C21" s="14" t="s">
         <v>119</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="E21" s="14" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="19" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C22" s="20" t="n">
         <v>5637</v>
@@ -27072,12 +27075,12 @@
         <v>0.20214444524134</v>
       </c>
       <c r="E22" s="19" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="19" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C23" s="20" t="n">
         <v>3913</v>
@@ -27087,12 +27090,12 @@
         <v>0.140321308183318</v>
       </c>
       <c r="E23" s="19" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="19" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C24" s="20" t="n">
         <v>3678</v>
@@ -27102,12 +27105,12 @@
         <v>0.131894140428889</v>
       </c>
       <c r="E24" s="19" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="19" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C25" s="20" t="n">
         <v>2744</v>
@@ -27117,12 +27120,12 @@
         <v>0.0984006311410744</v>
       </c>
       <c r="E25" s="23" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="19" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C26" s="20" t="n">
         <v>2071</v>
@@ -27132,12 +27135,12 @@
         <v>0.0742666571039231</v>
       </c>
       <c r="E26" s="19" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="19" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C27" s="20" t="n">
         <v>1937</v>
@@ -27147,12 +27150,12 @@
         <v>0.0694613784694829</v>
       </c>
       <c r="E27" s="19" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="19" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C28" s="20" t="n">
         <v>1726</v>
@@ -27162,12 +27165,12 @@
         <v>0.0618948576346554</v>
       </c>
       <c r="E28" s="19" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="19" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C29" s="20" t="n">
         <v>1029</v>
@@ -27177,12 +27180,12 @@
         <v>0.0369002366779029</v>
       </c>
       <c r="E29" s="19" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="19" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C30" s="20" t="n">
         <v>902</v>
@@ -27192,12 +27195,12 @@
         <v>0.0323459800616797</v>
       </c>
       <c r="E30" s="19" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="19" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C31" s="20" t="n">
         <v>612</v>
@@ -27207,12 +27210,12 @@
         <v>0.0219464964498315</v>
       </c>
       <c r="E31" s="19" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="19" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C32" s="20" t="n">
         <v>514</v>
@@ -27222,12 +27225,12 @@
         <v>0.0184321881947931</v>
       </c>
       <c r="E32" s="19" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="19" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C33" s="20" t="n">
         <v>501</v>
@@ -27237,12 +27240,12 @@
         <v>0.0179660044466758</v>
       </c>
       <c r="E33" s="23" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="19" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C34" s="20" t="n">
         <v>378</v>
@@ -27252,12 +27255,12 @@
         <v>0.0135551889837194</v>
       </c>
       <c r="E34" s="23" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="19" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C35" s="20" t="n">
         <v>335</v>
@@ -27267,12 +27270,12 @@
         <v>0.0120131965861006</v>
       </c>
       <c r="E35" s="19" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="19" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="C36" s="20" t="n">
         <v>333</v>
@@ -27282,12 +27285,12 @@
         <v>0.0119414760094671</v>
       </c>
       <c r="E36" s="23" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="19" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C37" s="20" t="n">
         <v>267</v>
@@ -27297,12 +27300,12 @@
         <v>0.00957469698056373</v>
       </c>
       <c r="E37" s="23" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="19" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C38" s="20" t="n">
         <v>260</v>
@@ -27312,12 +27315,12 @@
         <v>0.0093236749623467</v>
       </c>
       <c r="E38" s="19" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="19" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C39" s="20" t="n">
         <v>337</v>
@@ -27327,12 +27330,12 @@
         <v>0.012084917162734</v>
       </c>
       <c r="E39" s="23" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="19" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C40" s="20" t="n">
         <v>712</v>
@@ -27342,12 +27345,12 @@
         <v>0.0255325252815033</v>
       </c>
       <c r="E40" s="19" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="23" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="C41" s="24" t="n">
         <f aca="false">SUMIF(E22:E40,"BARISTA",C22:C40)</f>
@@ -27360,7 +27363,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="23" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C42" s="33" t="n">
         <f aca="false">C8-C41</f>
@@ -27373,7 +27376,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="14" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B44" s="14"/>
       <c r="C44" s="14"/>
@@ -27381,7 +27384,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="19" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C45" s="20" t="n">
         <f aca="false">C41*2</f>
@@ -27390,7 +27393,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="19" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C46" s="106" t="n">
         <v>0.5</v>
@@ -27398,7 +27401,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="19" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C47" s="20" t="n">
         <f aca="false">C45*C46</f>
@@ -27407,16 +27410,16 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="23" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C48" s="33" t="n">
-        <f aca="false">-C47*0.625</f>
-        <v>-2850</v>
+        <f aca="false">-C47*0.685</f>
+        <v>-3123.6</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="13" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C49" s="107" t="n">
         <v>0.25</v>
@@ -27433,25 +27436,25 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C50" s="20" t="n">
-        <f aca="false">-C45*0.25*0.625</f>
-        <v>-1425</v>
+        <f aca="false">-C45*0.25*0.685</f>
+        <v>-1561.8</v>
       </c>
       <c r="D50" s="20" t="n">
-        <f aca="false">-C45*0.5*0.625</f>
-        <v>-2850</v>
+        <f aca="false">-C45*0.5*0.685</f>
+        <v>-3123.6</v>
       </c>
       <c r="E50" s="20" t="n">
-        <f aca="false">-C45*0.75*0.625</f>
-        <v>-4275</v>
+        <f aca="false">-C45*0.75*0.685</f>
+        <v>-4685.4</v>
       </c>
       <c r="F50" s="20" t="n">
-        <f aca="false">-C45*1*0.625</f>
-        <v>-5700</v>
+        <f aca="false">-C45*1*0.685</f>
+        <v>-6247.2</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="14" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="B52" s="14"/>
       <c r="C52" s="14"/>
@@ -27459,7 +27462,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="19" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="C53" s="20" t="n">
         <v>2411</v>
@@ -27467,7 +27470,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="19" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="C54" s="20" t="n">
         <f aca="false">C53*2</f>
@@ -27476,7 +27479,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="13" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
     </row>
   </sheetData>
@@ -27510,7 +27513,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="108" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B1" s="37"/>
       <c r="C1" s="37"/>
@@ -27525,7 +27528,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="86" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="B2" s="86"/>
       <c r="C2" s="86"/>
@@ -27540,17 +27543,17 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="103" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B4" s="109" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="C4" s="110" t="n">
         <f aca="false">'LW Assumptions'!$C$23</f>
         <v>20</v>
       </c>
       <c r="D4" s="109" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="E4" s="110" t="n">
         <v>25</v>
@@ -27558,53 +27561,53 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="41" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="111" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="B7" s="111" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C7" s="112" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="D7" s="112" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="E7" s="112" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="F7" s="112" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="G7" s="112" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="H7" s="112" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="I7" s="112" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="J7" s="112" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="K7" s="112" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="L7" s="112" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="113" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="B8" s="114" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C8" s="115" t="n">
         <v>18.29</v>
@@ -27642,10 +27645,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="113" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="B9" s="114" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="C9" s="115" t="n">
         <v>21.03</v>
@@ -27682,15 +27685,15 @@
         <v>236.5875</v>
       </c>
       <c r="M9" s="120" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="113" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="B10" s="114" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C10" s="115" t="n">
         <v>17.79</v>
@@ -27729,10 +27732,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="113" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="B11" s="114" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="C11" s="115" t="n">
         <v>19.79</v>
@@ -27771,15 +27774,15 @@
         <v>692.65</v>
       </c>
       <c r="M11" s="120" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="113" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="B12" s="114" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="C12" s="115" t="n">
         <v>21.21</v>
@@ -27820,10 +27823,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="113" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="B13" s="114" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="C13" s="115" t="n">
         <v>25</v>
@@ -27859,12 +27862,12 @@
         <v>400</v>
       </c>
       <c r="M13" s="120" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="81" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="B14" s="87"/>
       <c r="C14" s="121"/>
@@ -27905,12 +27908,12 @@
         <v>2856.085</v>
       </c>
       <c r="M14" s="114" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="123" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B17" s="123"/>
       <c r="C17" s="123"/>
@@ -27926,36 +27929,36 @@
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="111"/>
       <c r="B18" s="111" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="D18" s="112" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="F18" s="112" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="G18" s="112" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="H18" s="112" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="J18" s="112" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="103" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="B19" s="113" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="D19" s="124" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="F19" s="125" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="G19" s="126" t="n">
         <v>8</v>
@@ -27972,13 +27975,13 @@
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="103"/>
       <c r="B20" s="113" t="s">
+        <v>453</v>
+      </c>
+      <c r="D20" s="124" t="s">
+        <v>454</v>
+      </c>
+      <c r="F20" s="125" t="s">
         <v>452</v>
-      </c>
-      <c r="D20" s="124" t="s">
-        <v>453</v>
-      </c>
-      <c r="F20" s="125" t="s">
-        <v>451</v>
       </c>
       <c r="G20" s="126" t="n">
         <v>8</v>
@@ -27995,13 +27998,13 @@
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="103"/>
       <c r="B21" s="113" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="D21" s="124" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="F21" s="125" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="G21" s="126" t="n">
         <v>4</v>
@@ -28017,7 +28020,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="127" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="B22" s="87"/>
       <c r="D22" s="87"/>
@@ -28037,18 +28040,18 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="127" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="B24" s="128" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C24" s="87"/>
       <c r="D24" s="129" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="E24" s="87"/>
       <c r="F24" s="130" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="G24" s="131" t="n">
         <v>10</v>
@@ -28066,15 +28069,15 @@
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="133"/>
       <c r="B25" s="134" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="C25" s="135"/>
       <c r="D25" s="136" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="E25" s="135"/>
       <c r="F25" s="137" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="G25" s="138" t="n">
         <v>0</v>
@@ -28090,7 +28093,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="127" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B26" s="87"/>
       <c r="D26" s="87"/>
@@ -28109,7 +28112,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="141" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="B28" s="141"/>
       <c r="C28" s="141"/>
@@ -28515,7 +28518,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="142" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="B1" s="37"/>
       <c r="C1" s="37"/>
@@ -28523,7 +28526,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="143" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="B2" s="143"/>
       <c r="C2" s="143"/>
@@ -28531,7 +28534,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="72" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="B4" s="42" t="s">
         <v>184</v>
@@ -28540,12 +28543,12 @@
         <v>185</v>
       </c>
       <c r="D4" s="42" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="43" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="B5" s="87"/>
       <c r="C5" s="87"/>
@@ -28553,7 +28556,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="88" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="B6" s="96" t="n">
         <v>119121</v>
@@ -28569,7 +28572,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="88" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="B7" s="96" t="n">
         <v>133545</v>
@@ -28585,7 +28588,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="88" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B8" s="96" t="n">
         <v>17887</v>
@@ -28601,7 +28604,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="88" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="B9" s="96" t="n">
         <v>6836</v>
@@ -28617,7 +28620,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="88" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B10" s="96" t="n">
         <v>-20307</v>
@@ -28633,7 +28636,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="88" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="B11" s="96" t="n">
         <v>1204</v>
@@ -28649,7 +28652,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="43" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B12" s="44" t="n">
         <v>258287</v>
@@ -28670,7 +28673,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="43" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="B14" s="147"/>
       <c r="C14" s="148"/>
@@ -28678,7 +28681,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="88" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="B15" s="96" t="n">
         <v>48655</v>
@@ -28694,7 +28697,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="88" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="B16" s="96" t="n">
         <v>27428</v>
@@ -28710,7 +28713,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="88" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B17" s="96" t="n">
         <v>5516</v>
@@ -28726,7 +28729,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="88" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B18" s="96" t="n">
         <v>0</v>
@@ -28742,7 +28745,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="43" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="B19" s="44" t="n">
         <v>81599</v>
@@ -28758,7 +28761,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="43" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="B20" s="44" t="n">
         <v>176688</v>
@@ -28787,7 +28790,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="88" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="B23" s="96" t="n">
         <v>142124</v>
@@ -28803,7 +28806,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="88" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="B24" s="96" t="n">
         <v>16219</v>
@@ -28819,7 +28822,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="88" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="B25" s="96" t="n">
         <v>6514</v>
@@ -28835,7 +28838,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="43" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="B26" s="44" t="n">
         <v>164857</v>
@@ -28856,7 +28859,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="43" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="B28" s="147"/>
       <c r="C28" s="148"/>
@@ -28864,7 +28867,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="88" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="B29" s="96" t="n">
         <v>44540</v>
@@ -28880,7 +28883,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="88" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="B30" s="96" t="n">
         <v>11918</v>
@@ -28896,7 +28899,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="88" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="B31" s="96" t="n">
         <v>2912</v>
@@ -28912,7 +28915,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="88" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="B32" s="96" t="n">
         <v>30305</v>
@@ -28928,7 +28931,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="43" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="B33" s="44" t="n">
         <v>89675</v>
@@ -28944,7 +28947,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="149" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B34" s="96" t="n">
         <v>10012</v>
@@ -28960,7 +28963,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="150" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="B35" s="74" t="n">
         <v>5657</v>
@@ -28976,7 +28979,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="151" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="B37" s="98" t="n">
         <v>-93513</v>
@@ -28992,7 +28995,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="88" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="B38" s="96" t="n">
         <v>-48000</v>
@@ -29004,7 +29007,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="88" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="B39" s="96" t="n">
         <v>-15642</v>
@@ -29016,7 +29019,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="151" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="B40" s="98" t="n">
         <v>-157155</v>
@@ -29032,7 +29035,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="153" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="B42" s="153"/>
       <c r="C42" s="153"/>
@@ -29074,7 +29077,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="85" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="B1" s="37"/>
       <c r="C1" s="37"/>
@@ -29087,7 +29090,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="86" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B2" s="86"/>
       <c r="C2" s="86"/>
@@ -29100,36 +29103,36 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="111" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="B4" s="111" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="C4" s="112" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="D4" s="112" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E4" s="112" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="F4" s="112" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="G4" s="112" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="H4" s="112" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="I4" s="112" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="154" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="B5" s="155"/>
       <c r="C5" s="156"/>
@@ -29142,10 +29145,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="113" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="B6" s="109" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="C6" s="157" t="n">
         <f aca="false">2441*12/5</f>
@@ -29177,10 +29180,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="113" t="s">
+        <v>518</v>
+      </c>
+      <c r="B7" s="109" t="s">
         <v>517</v>
-      </c>
-      <c r="B7" s="109" t="s">
-        <v>516</v>
       </c>
       <c r="C7" s="157" t="n">
         <f aca="false">1454*12/5</f>
@@ -29212,10 +29215,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="113" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="B8" s="109" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="C8" s="157" t="n">
         <f aca="false">823*12/5</f>
@@ -29247,10 +29250,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="113" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="B9" s="109" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="C9" s="157" t="n">
         <f aca="false">512*12/5</f>
@@ -29282,10 +29285,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="113" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="B10" s="109" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="C10" s="157" t="n">
         <f aca="false">528*12/5</f>
@@ -29317,10 +29320,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="113" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="B11" s="109" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="C11" s="157" t="n">
         <f aca="false">737*12/5</f>
@@ -29352,10 +29355,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="113" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="B12" s="109" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="C12" s="157" t="n">
         <f aca="false">348*12/5</f>
@@ -29387,10 +29390,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="113" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="B13" s="109" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="C13" s="157" t="n">
         <f aca="false">20731-SUM(C6:C12)</f>
@@ -29422,7 +29425,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="154" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="B14" s="155"/>
       <c r="C14" s="156"/>
@@ -29435,7 +29438,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="113" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="B15" s="109" t="s">
         <v>226</v>
@@ -29470,7 +29473,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="113" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="B16" s="109" t="s">
         <v>226</v>
@@ -29505,7 +29508,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="113" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="B17" s="109" t="s">
         <v>226</v>
@@ -29540,7 +29543,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="154" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="B18" s="155"/>
       <c r="C18" s="156"/>
@@ -29553,10 +29556,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="113" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="B19" s="109" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="C19" s="157" t="n">
         <f aca="false">385*12/5</f>
@@ -29588,10 +29591,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="113" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="B20" s="109" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="C20" s="157" t="n">
         <f aca="false">6022-C19</f>
@@ -29623,7 +29626,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="154" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B21" s="155"/>
       <c r="C21" s="155"/>
@@ -29636,7 +29639,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="113" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="B22" s="109" t="s">
         <v>226</v>
@@ -29669,10 +29672,10 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="113" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="B23" s="109" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="C23" s="157" t="n">
         <v>806</v>
@@ -29702,7 +29705,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="113" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="B24" s="109" t="s">
         <v>226</v>
@@ -29735,7 +29738,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="154" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="B25" s="155"/>
       <c r="C25" s="156"/>
@@ -29748,7 +29751,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="113" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="B26" s="109" t="s">
         <v>226</v>
@@ -29781,7 +29784,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="113" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="B27" s="109" t="s">
         <v>226</v>
@@ -29814,10 +29817,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="149" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="B28" s="109" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="C28" s="157" t="n">
         <v>358</v>
@@ -29847,7 +29850,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="81" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="B29" s="155"/>
       <c r="C29" s="165" t="n">
@@ -29872,7 +29875,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="109" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="B30" s="12"/>
       <c r="C30" s="18"/>
@@ -29896,7 +29899,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="123" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="B32" s="123"/>
       <c r="C32" s="123"/>
@@ -29909,7 +29912,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="65" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B33" s="12"/>
       <c r="C33" s="74" t="n">
@@ -29925,7 +29928,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="65" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="B34" s="12"/>
       <c r="C34" s="74" t="n">
@@ -29941,7 +29944,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="65" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="B35" s="12"/>
       <c r="C35" s="74" t="n">
@@ -29957,7 +29960,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="109" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="167" t="n">
@@ -29984,7 +29987,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="65" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="18"/>
@@ -29997,7 +30000,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="113" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="B39" s="12"/>
       <c r="C39" s="162" t="n">
@@ -30013,7 +30016,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="113" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="B40" s="12"/>
       <c r="C40" s="162" t="n">
@@ -30029,7 +30032,7 @@
     </row>
     <row r="41" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="168" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="B41" s="12"/>
       <c r="C41" s="162" t="n">
@@ -30056,7 +30059,7 @@
     </row>
     <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="170" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="B43" s="170"/>
       <c r="C43" s="170"/>
@@ -30069,7 +30072,7 @@
     </row>
     <row r="44" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="171" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="B44" s="171"/>
       <c r="C44" s="171"/>
@@ -30082,7 +30085,7 @@
     </row>
     <row r="45" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="171" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="B45" s="171"/>
       <c r="C45" s="171"/>
@@ -30095,7 +30098,7 @@
     </row>
     <row r="46" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="171" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="B46" s="171"/>
       <c r="C46" s="171"/>
@@ -30108,7 +30111,7 @@
     </row>
     <row r="47" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="171" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="B47" s="171"/>
       <c r="C47" s="171"/>
@@ -30121,7 +30124,7 @@
     </row>
     <row r="48" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="171" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="B48" s="171"/>
       <c r="C48" s="171"/>
@@ -30145,7 +30148,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="65" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="12"/>
@@ -30158,7 +30161,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="113" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="B51" s="12"/>
       <c r="C51" s="162" t="n">
@@ -30174,7 +30177,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="113" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="80" t="n">
@@ -30189,7 +30192,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="65" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="B53" s="12"/>
       <c r="C53" s="164" t="n">

</xml_diff>

<commit_message>
Relabel Vessel Assumptions: admin fee is income, not an owner charge
Input block relabeled so the 5% admin fee reads as client-billed
INCOME (to Other Operating Income) while mgmt fee/rent remain marked
as expenses. Labels only; no calculation changes.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VCQW3YoSqaJfwSKLPDyQy8
</commit_message>
<xml_diff>
--- a/Method_Operating_Model_2027_14.xlsx
+++ b/Method_Operating_Model_2027_14.xlsx
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1435" uniqueCount="562">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1435" uniqueCount="564">
   <si>
     <t xml:space="preserve">Method Terrapin</t>
   </si>
@@ -546,310 +546,316 @@
     <t xml:space="preserve">variable — own line</t>
   </si>
   <si>
-    <t xml:space="preserve">OWNER CHARGES  (above NOI)</t>
+    <t xml:space="preserve">OWNER CHARGES (above NOI) &amp; ADMIN FEE INCOME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Management fee (% of revenue) — EXPENSE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4% of gross revenue → Method (replaces profit split)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rent (% of revenue) — EXPENSE (waived)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vessel carries no separate rent (owner)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin fee (% of F&amp;B) — INCOME, billed to clients</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5% added to event client invoices → Vessel Other Operating Income (NOT an expense); 4% mgmt fee applies to it as revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Profit &amp; Loss Budget</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Events (2026 run-rate)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Events (budgeted, whole)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other Operating Income (svc charge + 5% admin fee)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin Fee (5% of F&amp;B — billed to clients, in income above)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beverage sales split across NA/Liquor/Beer/Wine pro-rata to the 2026 mix (uniform 25% beverage cost). Controllable lines distributed pro-rata to the Vessel 2026 P&amp;L. Net Operating Profit = model NOI (after 4% mgmt fee, 5% admin fee, rent $0).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VESSEL — GL COST BASIS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cost basis now linked to Vessel 2026 P&amp;L (Act/For) · controllable vs non-controllable (CC fees excluded)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Expense group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monthly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LABOR (in model)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Management labor – FOH mgmt (610300)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONTROLLABLE (excl credit card fees)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Direct operating (supplies, linen, equip)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G&amp;A / accounting / bank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marketing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Music &amp; entertainment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Repairs &amp; maintenance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total controllable (excl CC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">→ Controllable / month feed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NON-CONTROLLABLE (in model)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insurance – liability</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legal &amp; accounting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replacement reserves</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total non-controllable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VARIABLE / EXCLUDED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Credit card fees (actual GL → now variable 2.5%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Management fee (→ profit split)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rent / RE tax (owner)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Profit &amp; Loss Summary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Actual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forecast</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Act/For/Bud</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Little Wing Coffee &amp; Goods</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Profit &amp; Loss — 2026 Act/For MODIFIED · Jan–Jun actual, levers live from go-live date (staffing · pricing · retail · 4% fee)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 Modified</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Changes go-live date (INPUT):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">months on/after this date apply the levers; earlier months = unmodified Act/For</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fcst mod.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modified</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Retail / Merch Sales (new programming)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operating Expenses (incl CC on added rev)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modified months: single-shift staffing (FOH 6:30am–4pm + wknd 2nd barista, BOH cook $296/wk, GL mgmt labor kept), menu pricing uplift on Food/NA, retail uplift + programming on the Retail line (own COGS %), CC 2.5% on added revenue in OpEx, mgmt fee $4,000/mo → 4% of revenue, rent WAIVED (occupancy → 0%). All inputs on LW Assumptions / LW Menu Pricing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Profit &amp; Loss — 2026 Act/For MODIFIED · Jan–Jun actual, levers live from go-live date (4% mgmt fee · rent waived · 5% admin fee)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other Operating Income (svc charge + 5% admin fee when live)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modified months: management fee $4,000/mo → 4% of revenue, occupancy → 0% (waived), NEW 5% admin fee on F&amp;B billed to event clients — added to Other Operating Income (revenue), so the 4% mgmt fee also applies to it. Inputs on Vessel Assumptions C30–C32.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LITTLE WING  ·  COFFEE SHOP MODEL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Single-shift efficiency model — 6:30am–4pm operating hours (2nd barista Sat/Sun) + BOH cook kept, self-serve/retail after 4pm (front desk, no FOH labor)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REVENUE  (Toast H1 2026 actuals ×2 — Jan–Jun item detail, reconciled to Sales Summary)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Food</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NA / Coffee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">the margin engine — 22.2% cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alcohol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Retail / merch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gift cards, open items, uncategorized rings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL REVENUE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COST OF SALES  (% of each category · GL actual)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Food cost %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GL cost ÷ net sales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NA / Coffee cost %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alcohol cost %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Retail cost %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">no COGS booked in GL for retail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other cost %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">no COGS booked in GL for other</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADJUSTED LABOR  (single 6:30am–4pm shift + 2nd barista on peak days)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opener/supervisor hours/day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6:30am–4pm · one barista/supervisor (9.5h)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2nd barista avg hrs/day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sat &amp; Sun opener/closer overlap, 4 hrs/day ×2 days ÷7 — covers the 8–11a weekend rush</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Days per week</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blended wage $/hr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dolce actual blended FOH rate ~$20/hr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adjusted labor / year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">servers eliminated (self-serve); BOH cook KEPT at $296/wk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BOH cook labor — kept ($/wk base)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">current cook schedule held (~13.3 hrs/wk) — food program stays in-house</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CURRENT LABOR  (GL actual, for comparison)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Current labor / year (incl burden)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GL T12 actual: wages+taxes+benefits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VARIABLE &amp; OVERHEAD  (annual)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">go-forward target (Current column uses GL actual → C42)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Controllable exp (excl CC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">paper/plastics, accounting, linen…</t>
+  </si>
+  <si>
+    <t xml:space="preserve">insurance, legal, reserves</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RETAIL PROGRAMMING  (expanded merch/goods — new lever)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Retail programming — incremental revenue ($/yr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INPUT (placeholder ~$1K/mo) — new goods program layered on top of the existing-base uplift below</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Retail programming COGS %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">new merch carries real product cost (GL retail COGS was $0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BELOW NOI  (owner / occupancy)</t>
   </si>
   <si>
     <t xml:space="preserve">Management fee (% of revenue)</t>
   </si>
   <si>
-    <t xml:space="preserve">4% of gross revenue → Method (replaces profit split)</t>
+    <t xml:space="preserve">4% of gross revenue → Method (replaces $48K flat fee)</t>
   </si>
   <si>
     <t xml:space="preserve">Rent (% of revenue)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vessel carries no separate rent (owner)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Admin fee (% of F&amp;B revenue)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5% of food + beverage sales — billed to event clients (admin charge on the invoice) → Vessel Other Operating Income</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Profit &amp; Loss Budget</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Events (2026 run-rate)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Events (budgeted, whole)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Other Operating Income (svc charge + 5% admin fee)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Admin Fee (5% of F&amp;B — billed to clients, in income above)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Beverage sales split across NA/Liquor/Beer/Wine pro-rata to the 2026 mix (uniform 25% beverage cost). Controllable lines distributed pro-rata to the Vessel 2026 P&amp;L. Net Operating Profit = model NOI (after 4% mgmt fee, 5% admin fee, rent $0).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VESSEL — GL COST BASIS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cost basis now linked to Vessel 2026 P&amp;L (Act/For) · controllable vs non-controllable (CC fees excluded)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Expense group</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Annual</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Monthly</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LABOR (in model)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Management labor – FOH mgmt (610300)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CONTROLLABLE (excl credit card fees)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Direct operating (supplies, linen, equip)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G&amp;A / accounting / bank</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marketing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Music &amp; entertainment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Repairs &amp; maintenance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total controllable (excl CC)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">→ Controllable / month feed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NON-CONTROLLABLE (in model)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Insurance – liability</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Legal &amp; accounting</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replacement reserves</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total non-controllable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VARIABLE / EXCLUDED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Credit card fees (actual GL → now variable 2.5%)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Management fee (→ profit split)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rent / RE tax (owner)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Profit &amp; Loss Summary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Actual</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Forecast</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Act/For/Bud</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Little Wing Coffee &amp; Goods</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Profit &amp; Loss — 2026 Act/For MODIFIED · Jan–Jun actual, levers live from go-live date (staffing · pricing · retail · 4% fee)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 Modified</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Changes go-live date (INPUT):</t>
-  </si>
-  <si>
-    <t xml:space="preserve">months on/after this date apply the levers; earlier months = unmodified Act/For</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fcst mod.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modified</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Retail / Merch Sales (new programming)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Operating Expenses (incl CC on added rev)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modified months: single-shift staffing (FOH 6:30am–4pm + wknd 2nd barista, BOH cook $296/wk, GL mgmt labor kept), menu pricing uplift on Food/NA, retail uplift + programming on the Retail line (own COGS %), CC 2.5% on added revenue in OpEx, mgmt fee $4,000/mo → 4% of revenue, rent WAIVED (occupancy → 0%). All inputs on LW Assumptions / LW Menu Pricing.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Profit &amp; Loss — 2026 Act/For MODIFIED · Jan–Jun actual, levers live from go-live date (4% mgmt fee · rent waived · 5% admin fee)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Other Operating Income (svc charge + 5% admin fee when live)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modified months: management fee $4,000/mo → 4% of revenue, occupancy → 0% (waived), NEW 5% admin fee on F&amp;B billed to event clients — added to Other Operating Income (revenue), so the 4% mgmt fee also applies to it. Inputs on Vessel Assumptions C30–C32.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LITTLE WING  ·  COFFEE SHOP MODEL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Single-shift efficiency model — 6:30am–4pm operating hours (2nd barista Sat/Sun) + BOH cook kept, self-serve/retail after 4pm (front desk, no FOH labor)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REVENUE  (Toast H1 2026 actuals ×2 — Jan–Jun item detail, reconciled to Sales Summary)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Food</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NA / Coffee</t>
-  </si>
-  <si>
-    <t xml:space="preserve">the margin engine — 22.2% cost</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alcohol</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Retail / merch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Other</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gift cards, open items, uncategorized rings</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL REVENUE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COST OF SALES  (% of each category · GL actual)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Food cost %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GL cost ÷ net sales</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NA / Coffee cost %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alcohol cost %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Retail cost %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">no COGS booked in GL for retail</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Other cost %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">no COGS booked in GL for other</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADJUSTED LABOR  (single 6:30am–4pm shift + 2nd barista on peak days)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Opener/supervisor hours/day</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6:30am–4pm · one barista/supervisor (9.5h)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2nd barista avg hrs/day</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sat &amp; Sun opener/closer overlap, 4 hrs/day ×2 days ÷7 — covers the 8–11a weekend rush</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Days per week</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blended wage $/hr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dolce actual blended FOH rate ~$20/hr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adjusted labor / year</t>
-  </si>
-  <si>
-    <t xml:space="preserve">servers eliminated (self-serve); BOH cook KEPT at $296/wk</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BOH cook labor — kept ($/wk base)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">current cook schedule held (~13.3 hrs/wk) — food program stays in-house</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CURRENT LABOR  (GL actual, for comparison)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Current labor / year (incl burden)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GL T12 actual: wages+taxes+benefits</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VARIABLE &amp; OVERHEAD  (annual)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">go-forward target (Current column uses GL actual → C42)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Controllable exp (excl CC)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">paper/plastics, accounting, linen…</t>
-  </si>
-  <si>
-    <t xml:space="preserve">insurance, legal, reserves</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RETAIL PROGRAMMING  (expanded merch/goods — new lever)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Retail programming — incremental revenue ($/yr)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INPUT (placeholder ~$1K/mo) — new goods program layered on top of the existing-base uplift below</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Retail programming COGS %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">new merch carries real product cost (GL retail COGS was $0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BELOW NOI  (owner / occupancy)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4% of gross revenue → Method (replaces $48K flat fee)</t>
   </si>
   <si>
     <t xml:space="preserve">rent WAIVED (was 6% of revenue) — same treatment as Vessel; actuals keep booked occupancy</t>
@@ -19269,85 +19275,85 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="46" t="s">
-        <v>169</v>
+        <v>269</v>
       </c>
       <c r="C40" s="78" t="n">
         <v>0.04</v>
       </c>
       <c r="D40" s="62" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B41" s="46" t="s">
-        <v>171</v>
+        <v>271</v>
       </c>
       <c r="C41" s="78" t="n">
         <v>0</v>
       </c>
       <c r="D41" s="62" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B42" s="46" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="C42" s="44" t="n">
         <v>10012</v>
       </c>
       <c r="D42" s="62" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B43" s="46" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C43" s="44" t="n">
         <f aca="false">'LW Menu Pricing'!$C$53</f>
         <v>21617.37</v>
       </c>
       <c r="D43" s="62" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B44" s="46" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C44" s="79" t="n">
         <v>1</v>
       </c>
       <c r="D44" s="62" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B45" s="46" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C45" s="44" t="n">
         <v>12880</v>
       </c>
       <c r="D45" s="62" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B46" s="1" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C46" s="80" t="n">
         <v>0.5</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B47" s="1" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="C47" s="73" t="n">
         <f aca="false">'LW Assumptions'!$C$8*'LW Assumptions'!$C$46</f>
@@ -19402,7 +19408,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -19412,17 +19418,17 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C5" s="27" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="D5" s="27"/>
       <c r="E5" s="28"/>
       <c r="F5" s="27" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="G5" s="27"/>
       <c r="H5" s="28"/>
       <c r="I5" s="27" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="J5" s="27"/>
     </row>
@@ -20423,7 +20429,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="19" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="C54" s="20" t="n">
         <f aca="false">C20*0.06</f>
@@ -20788,7 +20794,7 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="13" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
   </sheetData>
@@ -20857,7 +20863,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26058,28 +26064,28 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="13" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="23" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="23" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="C75" s="23" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="E75" s="23" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="19" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="C76" s="71" t="n">
         <f aca="false">'LW Assumptions'!$C$20+'LW Assumptions'!$C$21</f>
@@ -26092,7 +26098,7 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="19" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C77" s="71" t="n">
         <v>8</v>
@@ -26104,7 +26110,7 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="19" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="C78" s="71" t="n">
         <v>13.5</v>
@@ -26116,7 +26122,7 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="19" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="C79" s="71" t="n">
         <v>16</v>
@@ -26185,7 +26191,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="39" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B1" s="39"/>
       <c r="C1" s="39"/>
@@ -26197,7 +26203,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="40" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B2" s="40"/>
       <c r="C2" s="40"/>
@@ -26209,35 +26215,35 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="41" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="F4" s="41" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="72" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="C5" s="42" t="s">
         <v>184</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="F5" s="72" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="G5" s="42" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="H5" s="42" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="46" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="C6" s="49" t="n">
         <v>42998</v>
@@ -26247,7 +26253,7 @@
         <v>0.161523943357004</v>
       </c>
       <c r="F6" s="46" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="G6" s="49" t="n">
         <v>72907</v>
@@ -26259,7 +26265,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="46" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="C7" s="49" t="n">
         <v>54634</v>
@@ -26269,7 +26275,7 @@
         <v>0.205235106780933</v>
       </c>
       <c r="F7" s="46" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="G7" s="49" t="n">
         <v>32396</v>
@@ -26281,7 +26287,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="46" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="C8" s="49" t="n">
         <v>30727</v>
@@ -26291,7 +26297,7 @@
         <v>0.115427373541343</v>
       </c>
       <c r="F8" s="81" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="G8" s="44" t="n">
         <f aca="false">G6+G7</f>
@@ -26304,7 +26310,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="46" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="C9" s="49" t="n">
         <v>12880</v>
@@ -26316,7 +26322,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="46" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="C10" s="49" t="n">
         <v>886</v>
@@ -26326,12 +26332,12 @@
         <v>0.00332829931192859</v>
       </c>
       <c r="F10" s="62" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="46" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="C11" s="49" t="n">
         <v>22733</v>
@@ -26341,12 +26347,12 @@
         <v>0.0853975488240097</v>
       </c>
       <c r="F11" s="62" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="81" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="C12" s="44" t="n">
         <f aca="false">SUM(C6:C11)</f>
@@ -26357,17 +26363,17 @@
         <v>0.619296577839642</v>
       </c>
       <c r="F12" s="62" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="41" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="46" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="C15" s="82" t="n">
         <f aca="false">'LW Assumptions'!C20+'LW Assumptions'!C21</f>
@@ -26376,7 +26382,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="46" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="C16" s="53" t="n">
         <f aca="false">('LW Assumptions'!C20+'LW Assumptions'!C21)*'LW Assumptions'!C22*52</f>
@@ -26385,7 +26391,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="46" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="C17" s="49" t="n">
         <f aca="false">C16*'LW Assumptions'!C23</f>
@@ -26394,7 +26400,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="46" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="C18" s="49" t="n">
         <f aca="false">'LW Assumptions'!C26*52</f>
@@ -26403,7 +26409,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="46" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="C19" s="49" t="n">
         <f aca="false">(C17+C18)*'LW Assumptions'!C24</f>
@@ -26412,7 +26418,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="46" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C20" s="53" t="n">
         <f aca="false">C17+C18+C19</f>
@@ -26421,7 +26427,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="83" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="C21" s="84" t="n">
         <f aca="false">C12-C20</f>
@@ -26430,7 +26436,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="59" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="C23" s="59"/>
       <c r="D23" s="59"/>
@@ -26479,7 +26485,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="85" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B1" s="37"/>
       <c r="C1" s="37"/>
@@ -26487,7 +26493,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="86" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B2" s="86"/>
       <c r="C2" s="86"/>
@@ -26496,18 +26502,18 @@
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="72"/>
       <c r="B4" s="42" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="C4" s="42" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="D4" s="42" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="81" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B5" s="87"/>
       <c r="C5" s="87"/>
@@ -26515,10 +26521,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="88" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B6" s="89" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="C6" s="89" t="n">
         <f aca="false">'LW Assumptions'!$C$20+'LW Assumptions'!$C$21</f>
@@ -26527,7 +26533,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="88" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B7" s="90" t="n">
         <v>7</v>
@@ -26539,7 +26545,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="81" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B9" s="87"/>
       <c r="C9" s="87"/>
@@ -26547,7 +26553,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="88" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B10" s="91" t="n">
         <v>111.8</v>
@@ -26559,7 +26565,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="88" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B11" s="91" t="n">
         <v>13.3</v>
@@ -26571,7 +26577,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="92" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B12" s="93" t="n">
         <v>125.1</v>
@@ -26588,7 +26594,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="81" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B14" s="87"/>
       <c r="C14" s="87"/>
@@ -26596,7 +26602,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="88" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B15" s="96" t="n">
         <v>2207</v>
@@ -26608,7 +26614,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="88" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B16" s="96" t="n">
         <v>296</v>
@@ -26620,7 +26626,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="94" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B17" s="74" t="n">
         <v>2503</v>
@@ -26632,7 +26638,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="88" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B18" s="96" t="n">
         <f aca="false">'LW Assumptions'!$C$45/52</f>
@@ -26645,7 +26651,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="88" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B19" s="96" t="n">
         <f aca="false">(B17+B18)*'LW Assumptions'!$C$24</f>
@@ -26658,7 +26664,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="97" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B20" s="98" t="n">
         <f aca="false">B17+B18+B19</f>
@@ -26681,7 +26687,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="94" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B22" s="74" t="n">
         <f aca="false">B20*52</f>
@@ -26704,7 +26710,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="81" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B24" s="87"/>
       <c r="C24" s="87"/>
@@ -26712,7 +26718,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="88" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B25" s="96" t="n">
         <v>5888.94</v>
@@ -26723,7 +26729,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="94" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B26" s="101" t="n">
         <f aca="false">B20/B25</f>
@@ -26746,7 +26752,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="102" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B28" s="102"/>
       <c r="C28" s="102"/>
@@ -26754,7 +26760,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="94" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="C29" s="74" t="n">
         <f aca="false">B20-C20</f>
@@ -26767,12 +26773,12 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="103" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="104" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B32" s="104"/>
       <c r="C32" s="104"/>
@@ -26786,12 +26792,12 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="103" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="104" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B36" s="104"/>
       <c r="C36" s="104"/>
@@ -26805,12 +26811,12 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="105" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="104" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B40" s="104"/>
       <c r="C40" s="104"/>
@@ -26861,24 +26867,24 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B4" s="14"/>
       <c r="C4" s="14" t="s">
         <v>119</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="C5" s="20" t="n">
         <v>2411</v>
@@ -26890,7 +26896,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="C6" s="20" t="n">
         <v>89592</v>
@@ -26902,7 +26908,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="C7" s="20" t="n">
         <v>13203</v>
@@ -26914,7 +26920,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="19" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="C8" s="33" t="n">
         <v>27886</v>
@@ -26926,7 +26932,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="23" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C9" s="24" t="n">
         <f aca="false">SUM(C5:C8)</f>
@@ -26935,22 +26941,22 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B12" s="14"/>
       <c r="C12" s="14" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27045,27 +27051,27 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="14" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B21" s="14"/>
       <c r="C21" s="14" t="s">
         <v>119</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="E21" s="14" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="19" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="C22" s="20" t="n">
         <v>5637</v>
@@ -27075,12 +27081,12 @@
         <v>0.20214444524134</v>
       </c>
       <c r="E22" s="19" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="19" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="C23" s="20" t="n">
         <v>3913</v>
@@ -27090,12 +27096,12 @@
         <v>0.140321308183318</v>
       </c>
       <c r="E23" s="19" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="19" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="C24" s="20" t="n">
         <v>3678</v>
@@ -27105,12 +27111,12 @@
         <v>0.131894140428889</v>
       </c>
       <c r="E24" s="19" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="19" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="C25" s="20" t="n">
         <v>2744</v>
@@ -27120,12 +27126,12 @@
         <v>0.0984006311410744</v>
       </c>
       <c r="E25" s="23" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="19" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="C26" s="20" t="n">
         <v>2071</v>
@@ -27135,12 +27141,12 @@
         <v>0.0742666571039231</v>
       </c>
       <c r="E26" s="19" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="19" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="C27" s="20" t="n">
         <v>1937</v>
@@ -27150,12 +27156,12 @@
         <v>0.0694613784694829</v>
       </c>
       <c r="E27" s="19" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="19" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="C28" s="20" t="n">
         <v>1726</v>
@@ -27165,12 +27171,12 @@
         <v>0.0618948576346554</v>
       </c>
       <c r="E28" s="19" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="19" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="C29" s="20" t="n">
         <v>1029</v>
@@ -27180,12 +27186,12 @@
         <v>0.0369002366779029</v>
       </c>
       <c r="E29" s="19" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="19" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="C30" s="20" t="n">
         <v>902</v>
@@ -27195,12 +27201,12 @@
         <v>0.0323459800616797</v>
       </c>
       <c r="E30" s="19" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="19" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="C31" s="20" t="n">
         <v>612</v>
@@ -27210,12 +27216,12 @@
         <v>0.0219464964498315</v>
       </c>
       <c r="E31" s="19" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="19" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="C32" s="20" t="n">
         <v>514</v>
@@ -27225,12 +27231,12 @@
         <v>0.0184321881947931</v>
       </c>
       <c r="E32" s="19" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="19" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="C33" s="20" t="n">
         <v>501</v>
@@ -27240,12 +27246,12 @@
         <v>0.0179660044466758</v>
       </c>
       <c r="E33" s="23" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="19" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="C34" s="20" t="n">
         <v>378</v>
@@ -27255,12 +27261,12 @@
         <v>0.0135551889837194</v>
       </c>
       <c r="E34" s="23" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="19" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="C35" s="20" t="n">
         <v>335</v>
@@ -27270,12 +27276,12 @@
         <v>0.0120131965861006</v>
       </c>
       <c r="E35" s="19" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="19" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="C36" s="20" t="n">
         <v>333</v>
@@ -27285,12 +27291,12 @@
         <v>0.0119414760094671</v>
       </c>
       <c r="E36" s="23" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="19" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="C37" s="20" t="n">
         <v>267</v>
@@ -27300,12 +27306,12 @@
         <v>0.00957469698056373</v>
       </c>
       <c r="E37" s="23" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="19" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="C38" s="20" t="n">
         <v>260</v>
@@ -27315,12 +27321,12 @@
         <v>0.0093236749623467</v>
       </c>
       <c r="E38" s="19" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="19" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="C39" s="20" t="n">
         <v>337</v>
@@ -27330,12 +27336,12 @@
         <v>0.012084917162734</v>
       </c>
       <c r="E39" s="23" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="19" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="C40" s="20" t="n">
         <v>712</v>
@@ -27345,12 +27351,12 @@
         <v>0.0255325252815033</v>
       </c>
       <c r="E40" s="19" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="23" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="C41" s="24" t="n">
         <f aca="false">SUMIF(E22:E40,"BARISTA",C22:C40)</f>
@@ -27363,7 +27369,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="23" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="C42" s="33" t="n">
         <f aca="false">C8-C41</f>
@@ -27376,7 +27382,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="14" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B44" s="14"/>
       <c r="C44" s="14"/>
@@ -27384,7 +27390,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="19" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="C45" s="20" t="n">
         <f aca="false">C41*2</f>
@@ -27393,7 +27399,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="19" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="C46" s="106" t="n">
         <v>0.5</v>
@@ -27401,7 +27407,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="19" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="C47" s="20" t="n">
         <f aca="false">C45*C46</f>
@@ -27410,7 +27416,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="23" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="C48" s="33" t="n">
         <f aca="false">-C47*0.685</f>
@@ -27419,7 +27425,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="13" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="C49" s="107" t="n">
         <v>0.25</v>
@@ -27454,7 +27460,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="14" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B52" s="14"/>
       <c r="C52" s="14"/>
@@ -27462,7 +27468,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="19" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="C53" s="20" t="n">
         <v>2411</v>
@@ -27470,7 +27476,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="19" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="C54" s="20" t="n">
         <f aca="false">C53*2</f>
@@ -27479,7 +27485,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="13" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
     </row>
   </sheetData>
@@ -27513,7 +27519,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="108" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B1" s="37"/>
       <c r="C1" s="37"/>
@@ -27528,7 +27534,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="86" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B2" s="86"/>
       <c r="C2" s="86"/>
@@ -27543,17 +27549,17 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="103" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B4" s="109" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="C4" s="110" t="n">
         <f aca="false">'LW Assumptions'!$C$23</f>
         <v>20</v>
       </c>
       <c r="D4" s="109" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="E4" s="110" t="n">
         <v>25</v>
@@ -27561,53 +27567,53 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="41" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="111" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B7" s="111" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="C7" s="112" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="D7" s="112" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="E7" s="112" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="F7" s="112" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="G7" s="112" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="H7" s="112" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="I7" s="112" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="J7" s="112" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="K7" s="112" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="L7" s="112" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="113" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B8" s="114" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="C8" s="115" t="n">
         <v>18.29</v>
@@ -27645,10 +27651,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="113" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B9" s="114" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="C9" s="115" t="n">
         <v>21.03</v>
@@ -27685,15 +27691,15 @@
         <v>236.5875</v>
       </c>
       <c r="M9" s="120" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="113" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B10" s="114" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="C10" s="115" t="n">
         <v>17.79</v>
@@ -27732,10 +27738,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="113" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B11" s="114" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="C11" s="115" t="n">
         <v>19.79</v>
@@ -27774,15 +27780,15 @@
         <v>692.65</v>
       </c>
       <c r="M11" s="120" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="113" t="s">
+        <v>438</v>
+      </c>
+      <c r="B12" s="114" t="s">
         <v>436</v>
-      </c>
-      <c r="B12" s="114" t="s">
-        <v>434</v>
       </c>
       <c r="C12" s="115" t="n">
         <v>21.21</v>
@@ -27823,10 +27829,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="113" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B13" s="114" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="C13" s="115" t="n">
         <v>25</v>
@@ -27862,12 +27868,12 @@
         <v>400</v>
       </c>
       <c r="M13" s="120" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="81" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B14" s="87"/>
       <c r="C14" s="121"/>
@@ -27908,12 +27914,12 @@
         <v>2856.085</v>
       </c>
       <c r="M14" s="114" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="123" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B17" s="123"/>
       <c r="C17" s="123"/>
@@ -27929,36 +27935,36 @@
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="111"/>
       <c r="B18" s="111" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="D18" s="112" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="F18" s="112" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="G18" s="112" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="H18" s="112" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="J18" s="112" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="103" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B19" s="113" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="D19" s="124" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="F19" s="125" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="G19" s="126" t="n">
         <v>8</v>
@@ -27975,13 +27981,13 @@
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="103"/>
       <c r="B20" s="113" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="D20" s="124" t="s">
+        <v>456</v>
+      </c>
+      <c r="F20" s="125" t="s">
         <v>454</v>
-      </c>
-      <c r="F20" s="125" t="s">
-        <v>452</v>
       </c>
       <c r="G20" s="126" t="n">
         <v>8</v>
@@ -27998,13 +28004,13 @@
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="103"/>
       <c r="B21" s="113" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="D21" s="124" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="F21" s="125" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="G21" s="126" t="n">
         <v>4</v>
@@ -28020,7 +28026,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="127" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="B22" s="87"/>
       <c r="D22" s="87"/>
@@ -28040,18 +28046,18 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="127" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B24" s="128" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="C24" s="87"/>
       <c r="D24" s="129" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="E24" s="87"/>
       <c r="F24" s="130" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="G24" s="131" t="n">
         <v>10</v>
@@ -28069,15 +28075,15 @@
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="133"/>
       <c r="B25" s="134" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="C25" s="135"/>
       <c r="D25" s="136" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="E25" s="135"/>
       <c r="F25" s="137" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="G25" s="138" t="n">
         <v>0</v>
@@ -28093,7 +28099,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="127" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="B26" s="87"/>
       <c r="D26" s="87"/>
@@ -28112,7 +28118,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="141" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B28" s="141"/>
       <c r="C28" s="141"/>
@@ -28518,7 +28524,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="142" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B1" s="37"/>
       <c r="C1" s="37"/>
@@ -28526,7 +28532,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="143" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="B2" s="143"/>
       <c r="C2" s="143"/>
@@ -28534,7 +28540,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="72" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B4" s="42" t="s">
         <v>184</v>
@@ -28543,12 +28549,12 @@
         <v>185</v>
       </c>
       <c r="D4" s="42" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="43" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B5" s="87"/>
       <c r="C5" s="87"/>
@@ -28556,7 +28562,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="88" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="B6" s="96" t="n">
         <v>119121</v>
@@ -28572,7 +28578,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="88" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="B7" s="96" t="n">
         <v>133545</v>
@@ -28588,7 +28594,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="88" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B8" s="96" t="n">
         <v>17887</v>
@@ -28604,7 +28610,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="88" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="B9" s="96" t="n">
         <v>6836</v>
@@ -28620,7 +28626,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="88" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="B10" s="96" t="n">
         <v>-20307</v>
@@ -28636,7 +28642,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="88" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="B11" s="96" t="n">
         <v>1204</v>
@@ -28652,7 +28658,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="43" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B12" s="44" t="n">
         <v>258287</v>
@@ -28673,7 +28679,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="43" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B14" s="147"/>
       <c r="C14" s="148"/>
@@ -28681,7 +28687,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="88" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B15" s="96" t="n">
         <v>48655</v>
@@ -28697,7 +28703,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="88" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="B16" s="96" t="n">
         <v>27428</v>
@@ -28713,7 +28719,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="88" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B17" s="96" t="n">
         <v>5516</v>
@@ -28729,7 +28735,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="88" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="B18" s="96" t="n">
         <v>0</v>
@@ -28745,7 +28751,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="43" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="B19" s="44" t="n">
         <v>81599</v>
@@ -28761,7 +28767,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="43" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="B20" s="44" t="n">
         <v>176688</v>
@@ -28790,7 +28796,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="88" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B23" s="96" t="n">
         <v>142124</v>
@@ -28806,7 +28812,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="88" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="B24" s="96" t="n">
         <v>16219</v>
@@ -28822,7 +28828,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="88" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="B25" s="96" t="n">
         <v>6514</v>
@@ -28838,7 +28844,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="43" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B26" s="44" t="n">
         <v>164857</v>
@@ -28859,7 +28865,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="43" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="B28" s="147"/>
       <c r="C28" s="148"/>
@@ -28867,7 +28873,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="88" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="B29" s="96" t="n">
         <v>44540</v>
@@ -28883,7 +28889,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="88" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="B30" s="96" t="n">
         <v>11918</v>
@@ -28899,7 +28905,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="88" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B31" s="96" t="n">
         <v>2912</v>
@@ -28915,7 +28921,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="88" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="B32" s="96" t="n">
         <v>30305</v>
@@ -28931,7 +28937,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="43" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="B33" s="44" t="n">
         <v>89675</v>
@@ -28947,7 +28953,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="149" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="B34" s="96" t="n">
         <v>10012</v>
@@ -28963,7 +28969,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="150" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="B35" s="74" t="n">
         <v>5657</v>
@@ -28979,7 +28985,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="151" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="B37" s="98" t="n">
         <v>-93513</v>
@@ -28995,7 +29001,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="88" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="B38" s="96" t="n">
         <v>-48000</v>
@@ -29007,7 +29013,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="88" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="B39" s="96" t="n">
         <v>-15642</v>
@@ -29019,7 +29025,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="151" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="B40" s="98" t="n">
         <v>-157155</v>
@@ -29035,7 +29041,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="153" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="B42" s="153"/>
       <c r="C42" s="153"/>
@@ -29077,7 +29083,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="85" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="B1" s="37"/>
       <c r="C1" s="37"/>
@@ -29090,7 +29096,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="86" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="B2" s="86"/>
       <c r="C2" s="86"/>
@@ -29103,36 +29109,36 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="111" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="B4" s="111" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="C4" s="112" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="D4" s="112" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="E4" s="112" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="F4" s="112" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="G4" s="112" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="H4" s="112" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="I4" s="112" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="154" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B5" s="155"/>
       <c r="C5" s="156"/>
@@ -29145,10 +29151,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="113" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B6" s="109" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="C6" s="157" t="n">
         <f aca="false">2441*12/5</f>
@@ -29180,10 +29186,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="113" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="B7" s="109" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="C7" s="157" t="n">
         <f aca="false">1454*12/5</f>
@@ -29215,10 +29221,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="113" t="s">
+        <v>521</v>
+      </c>
+      <c r="B8" s="109" t="s">
         <v>519</v>
-      </c>
-      <c r="B8" s="109" t="s">
-        <v>517</v>
       </c>
       <c r="C8" s="157" t="n">
         <f aca="false">823*12/5</f>
@@ -29250,10 +29256,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="113" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="B9" s="109" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="C9" s="157" t="n">
         <f aca="false">512*12/5</f>
@@ -29285,10 +29291,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="113" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="B10" s="109" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="C10" s="157" t="n">
         <f aca="false">528*12/5</f>
@@ -29320,10 +29326,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="113" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B11" s="109" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="C11" s="157" t="n">
         <f aca="false">737*12/5</f>
@@ -29355,10 +29361,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="113" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="B12" s="109" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="C12" s="157" t="n">
         <f aca="false">348*12/5</f>
@@ -29390,10 +29396,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="113" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="B13" s="109" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="C13" s="157" t="n">
         <f aca="false">20731-SUM(C6:C12)</f>
@@ -29425,7 +29431,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="154" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="B14" s="155"/>
       <c r="C14" s="156"/>
@@ -29438,7 +29444,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="113" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="B15" s="109" t="s">
         <v>226</v>
@@ -29473,7 +29479,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="113" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="B16" s="109" t="s">
         <v>226</v>
@@ -29508,7 +29514,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="113" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="B17" s="109" t="s">
         <v>226</v>
@@ -29543,7 +29549,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="154" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="B18" s="155"/>
       <c r="C18" s="156"/>
@@ -29556,10 +29562,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="113" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="B19" s="109" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="C19" s="157" t="n">
         <f aca="false">385*12/5</f>
@@ -29591,10 +29597,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="113" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="B20" s="109" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="C20" s="157" t="n">
         <f aca="false">6022-C19</f>
@@ -29626,7 +29632,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="154" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="B21" s="155"/>
       <c r="C21" s="155"/>
@@ -29639,7 +29645,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="113" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="B22" s="109" t="s">
         <v>226</v>
@@ -29672,10 +29678,10 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="113" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="B23" s="109" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="C23" s="157" t="n">
         <v>806</v>
@@ -29705,7 +29711,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="113" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="B24" s="109" t="s">
         <v>226</v>
@@ -29738,7 +29744,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="154" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="B25" s="155"/>
       <c r="C25" s="156"/>
@@ -29751,7 +29757,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="113" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="B26" s="109" t="s">
         <v>226</v>
@@ -29784,7 +29790,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="113" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="B27" s="109" t="s">
         <v>226</v>
@@ -29817,10 +29823,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="149" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="B28" s="109" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="C28" s="157" t="n">
         <v>358</v>
@@ -29850,7 +29856,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="81" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="B29" s="155"/>
       <c r="C29" s="165" t="n">
@@ -29875,7 +29881,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="109" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="B30" s="12"/>
       <c r="C30" s="18"/>
@@ -29899,7 +29905,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="123" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="B32" s="123"/>
       <c r="C32" s="123"/>
@@ -29912,7 +29918,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="65" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="B33" s="12"/>
       <c r="C33" s="74" t="n">
@@ -29928,7 +29934,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="65" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="B34" s="12"/>
       <c r="C34" s="74" t="n">
@@ -29944,7 +29950,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="65" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="B35" s="12"/>
       <c r="C35" s="74" t="n">
@@ -29960,7 +29966,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="109" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="167" t="n">
@@ -29987,7 +29993,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="65" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="18"/>
@@ -30000,7 +30006,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="113" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="B39" s="12"/>
       <c r="C39" s="162" t="n">
@@ -30016,7 +30022,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="113" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="B40" s="12"/>
       <c r="C40" s="162" t="n">
@@ -30032,7 +30038,7 @@
     </row>
     <row r="41" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="168" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="B41" s="12"/>
       <c r="C41" s="162" t="n">
@@ -30059,7 +30065,7 @@
     </row>
     <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="170" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="B43" s="170"/>
       <c r="C43" s="170"/>
@@ -30072,7 +30078,7 @@
     </row>
     <row r="44" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="171" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="B44" s="171"/>
       <c r="C44" s="171"/>
@@ -30085,7 +30091,7 @@
     </row>
     <row r="45" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="171" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="B45" s="171"/>
       <c r="C45" s="171"/>
@@ -30098,7 +30104,7 @@
     </row>
     <row r="46" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="171" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="B46" s="171"/>
       <c r="C46" s="171"/>
@@ -30111,7 +30117,7 @@
     </row>
     <row r="47" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="171" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="B47" s="171"/>
       <c r="C47" s="171"/>
@@ -30124,7 +30130,7 @@
     </row>
     <row r="48" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="171" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="B48" s="171"/>
       <c r="C48" s="171"/>
@@ -30148,7 +30154,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="65" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="12"/>
@@ -30161,7 +30167,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="113" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="B51" s="12"/>
       <c r="C51" s="162" t="n">
@@ -30177,7 +30183,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="113" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="80" t="n">
@@ -30192,7 +30198,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="65" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="B53" s="12"/>
       <c r="C53" s="164" t="n">

</xml_diff>